<commit_message>
Se ajusta la app de la clase 5 v2
</commit_message>
<xml_diff>
--- a/FundProg/Notas/Notas_FundProg.xlsx
+++ b/FundProg/Notas/Notas_FundProg.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E18DF12-E2AC-4DE8-B9DE-3DDCAD7936E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E134CB-BDB7-4FF3-B7FF-E72CD69402C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="report name" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
     <sheet name="Quiz 1_Consolidado" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'report name'!$D$1:$E$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'report name'!$A$1:$J$31</definedName>
     <definedName name="JR_PAGE_ANCHOR_0_1" localSheetId="1">Q1_V1!#REF!</definedName>
     <definedName name="JR_PAGE_ANCHOR_0_1" localSheetId="2">Q1_V2!#REF!</definedName>
     <definedName name="JR_PAGE_ANCHOR_0_1" localSheetId="3">Q1_V3!#REF!</definedName>
@@ -38,8 +38,66 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Autor</author>
+  </authors>
+  <commentList>
+    <comment ref="H18" authorId="0" shapeId="0" xr:uid="{2A3EE87D-F3EF-4EE9-A367-23E5D67270AF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Autor:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+No vino a la clase, tiene falta ese día</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I18" authorId="0" shapeId="0" xr:uid="{2DD9E89D-07A6-46AB-826F-66C07B4AFC34}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Autor:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+No vino a la clase</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="52">
   <si>
     <t>Porcentaje</t>
   </si>
@@ -172,6 +230,30 @@
   <si>
     <t>DDD</t>
   </si>
+  <si>
+    <t>Taller 1</t>
+  </si>
+  <si>
+    <t>Taller 2</t>
+  </si>
+  <si>
+    <t>Taller 3</t>
+  </si>
+  <si>
+    <t>Taller 4</t>
+  </si>
+  <si>
+    <t>Promedio</t>
+  </si>
+  <si>
+    <t>hizo 5 de 6</t>
+  </si>
+  <si>
+    <t>Definitiva</t>
+  </si>
+  <si>
+    <t>ss</t>
+  </si>
 </sst>
 </file>
 
@@ -182,7 +264,7 @@
     <numFmt numFmtId="165" formatCode="0.00000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,6 +296,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -290,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -316,9 +411,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -330,6 +422,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -353,13 +454,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -396,13 +497,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -439,13 +540,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -482,13 +583,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -525,13 +626,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -568,13 +669,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -611,13 +712,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -654,16 +755,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -697,16 +798,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -740,13 +841,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -783,13 +884,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -826,13 +927,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -869,13 +970,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -912,13 +1013,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -955,16 +1056,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -998,16 +1099,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1041,16 +1142,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1084,16 +1185,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1127,16 +1228,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1170,16 +1271,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1213,13 +1314,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1256,13 +1357,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1299,13 +1400,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1342,13 +1443,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1385,13 +1486,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1428,13 +1529,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1471,13 +1572,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1514,13 +1615,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1557,13 +1658,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1600,13 +1701,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1643,13 +1744,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1686,13 +1787,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -1729,16 +1830,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1772,16 +1873,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1815,16 +1916,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1858,16 +1959,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1901,16 +2002,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1944,16 +2045,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1987,16 +2088,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2030,16 +2131,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2073,16 +2174,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2116,16 +2217,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2159,16 +2260,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2202,16 +2303,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2245,13 +2346,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2288,13 +2389,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2331,13 +2432,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2374,13 +2475,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2417,13 +2518,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2460,13 +2561,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2503,13 +2604,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2546,13 +2647,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2589,13 +2690,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2632,13 +2733,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2675,13 +2776,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2718,13 +2819,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -2761,13 +2862,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -2804,13 +2905,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -2847,13 +2948,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -2890,13 +2991,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -2933,13 +3034,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -2976,13 +3077,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -3019,13 +3120,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3062,13 +3163,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3105,13 +3206,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3148,13 +3249,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3191,13 +3292,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3234,13 +3335,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3277,13 +3378,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3320,13 +3421,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3363,13 +3464,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3406,13 +3507,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3449,13 +3550,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3492,13 +3593,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3535,13 +3636,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3578,13 +3679,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3621,13 +3722,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3664,13 +3765,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3707,13 +3808,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3750,13 +3851,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3793,13 +3894,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3836,13 +3937,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3879,13 +3980,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3922,13 +4023,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -3965,13 +4066,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -4008,16 +4109,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4051,16 +4152,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4094,16 +4195,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4137,16 +4238,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4180,16 +4281,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4223,16 +4324,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4266,13 +4367,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -4309,13 +4410,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -4352,13 +4453,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -4395,13 +4496,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -4438,13 +4539,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -4481,13 +4582,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -4524,16 +4625,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4567,16 +4668,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4610,16 +4711,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4653,16 +4754,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4696,16 +4797,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4739,16 +4840,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4782,13 +4883,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -4825,13 +4926,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -4868,13 +4969,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -4911,13 +5012,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -4954,13 +5055,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -4997,13 +5098,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -5040,16 +5141,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5083,16 +5184,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5126,16 +5227,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5169,16 +5270,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5212,16 +5313,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5255,16 +5356,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>512</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5298,16 +5399,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>8255</xdr:rowOff>
+      <xdr:rowOff>19685</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5341,16 +5442,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>359410</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>8255</xdr:rowOff>
+      <xdr:rowOff>19685</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5384,16 +5485,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>8255</xdr:rowOff>
+      <xdr:rowOff>19685</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5427,16 +5528,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>8255</xdr:rowOff>
+      <xdr:rowOff>19685</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5470,16 +5571,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>8255</xdr:rowOff>
+      <xdr:rowOff>19685</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5513,16 +5614,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>8255</xdr:rowOff>
+      <xdr:rowOff>19685</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5556,13 +5657,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>58420</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>15875</xdr:rowOff>
@@ -5599,13 +5700,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>24</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>361315</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>635</xdr:rowOff>
@@ -21841,43 +21942,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:X31"/>
+  <dimension ref="A1:AE31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.33203125" customWidth="1"/>
-    <col min="2" max="24" width="11.6640625" customWidth="1"/>
+    <col min="2" max="31" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="31.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" ht="31.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
+      <c r="C1" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="D1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="J1" s="4" t="s">
+        <v>50</v>
+      </c>
       <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
+      <c r="L1" s="4" t="s">
+        <v>51</v>
+      </c>
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="O1" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
+      <c r="Q1" s="8">
+        <f>(5/6)*5</f>
+        <v>4.166666666666667</v>
+      </c>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
       <c r="T1" s="4"/>
@@ -21885,35 +22005,55 @@
       <c r="V1" s="4"/>
       <c r="W1" s="4"/>
       <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="4"/>
+      <c r="AA1" s="4"/>
+      <c r="AB1" s="4"/>
+      <c r="AC1" s="4"/>
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
     </row>
-    <row r="2" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3">
         <v>0</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="9">
+      <c r="C2" s="8">
+        <v>5</v>
+      </c>
+      <c r="D2" s="8">
+        <v>5</v>
+      </c>
+      <c r="E2" s="8">
+        <v>5</v>
+      </c>
+      <c r="F2" s="8">
+        <v>4</v>
+      </c>
+      <c r="G2" s="9">
+        <f>AVERAGE(C2:F2)</f>
+        <v>4.75</v>
+      </c>
+      <c r="H2" s="9">
         <f>VLOOKUP(A2,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>4.38</v>
       </c>
-      <c r="E2" s="8">
+      <c r="I2" s="8">
         <v>4.38</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4" t="e">
-        <f>AVERAGE(D2:D31)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="J2" s="9">
+        <f>G2*0.4+H2*0.6</f>
+        <v>4.5279999999999996</v>
+      </c>
       <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
+      <c r="L2" s="8">
+        <f>IF(G2&lt;J2,1,0)</f>
+        <v>0</v>
+      </c>
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
@@ -21923,29 +22063,53 @@
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
+      <c r="AA2" s="4"/>
+      <c r="AB2" s="4"/>
+      <c r="AC2" s="4"/>
+      <c r="AD2" s="4"/>
+      <c r="AE2" s="4"/>
     </row>
-    <row r="3" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="16" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="3">
         <v>0</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="9">
+      <c r="C3" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D3" s="8">
+        <v>3</v>
+      </c>
+      <c r="E3" s="8">
+        <v>5</v>
+      </c>
+      <c r="F3" s="8">
+        <v>4</v>
+      </c>
+      <c r="G3" s="9">
+        <f t="shared" ref="G3:G31" si="0">AVERAGE(C3:F3)</f>
+        <v>4.05</v>
+      </c>
+      <c r="H3" s="9">
         <f>VLOOKUP(A3,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>1.9900000000000002</v>
       </c>
-      <c r="E3" s="9">
+      <c r="I3" s="9">
         <v>1.9900000000000002</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
+      <c r="J3" s="9">
+        <f t="shared" ref="J3:J31" si="1">G3*0.4+H3*0.6</f>
+        <v>2.8140000000000001</v>
+      </c>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+      <c r="L3" s="8">
+        <f t="shared" ref="L3:L31" si="2">IF(G3&lt;J3,1,0)</f>
+        <v>0</v>
+      </c>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
@@ -21958,64 +22122,112 @@
       <c r="V3" s="4"/>
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
     </row>
-    <row r="4" spans="1:24" s="15" customFormat="1" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:31" s="14" customFormat="1" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>0.3125</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="14" t="e">
+      <c r="C4" s="15">
+        <v>0</v>
+      </c>
+      <c r="D4" s="15">
+        <v>0</v>
+      </c>
+      <c r="E4" s="15">
+        <v>0</v>
+      </c>
+      <c r="F4" s="15">
+        <v>0</v>
+      </c>
+      <c r="G4" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H4" s="13" t="e">
         <f>VLOOKUP(A4,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>#N/A</v>
       </c>
-      <c r="E4" s="16" t="e">
+      <c r="I4" s="15" t="e">
         <v>#N/A</v>
       </c>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
-      <c r="V4" s="13"/>
-      <c r="W4" s="13"/>
-      <c r="X4" s="13"/>
+      <c r="J4" s="13" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="K4" s="12"/>
+      <c r="L4" s="8" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
+      <c r="AB4" s="12"/>
+      <c r="AC4" s="12"/>
+      <c r="AD4" s="12"/>
+      <c r="AE4" s="12"/>
     </row>
-    <row r="5" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="16" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="3">
         <v>0</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="9">
+      <c r="C5" s="8">
+        <v>5</v>
+      </c>
+      <c r="D5" s="8">
+        <v>5</v>
+      </c>
+      <c r="E5" s="8">
+        <v>5</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0</v>
+      </c>
+      <c r="G5" s="9">
+        <f t="shared" si="0"/>
+        <v>3.75</v>
+      </c>
+      <c r="H5" s="9">
         <f>VLOOKUP(A5,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>2.62</v>
       </c>
-      <c r="E5" s="9">
+      <c r="I5" s="9">
         <v>2.62</v>
       </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
+      <c r="J5" s="9">
+        <f t="shared" si="1"/>
+        <v>3.0720000000000001</v>
+      </c>
       <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="L5" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
@@ -22028,29 +22240,53 @@
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="4"/>
+      <c r="AB5" s="4"/>
+      <c r="AC5" s="4"/>
+      <c r="AD5" s="4"/>
+      <c r="AE5" s="4"/>
     </row>
-    <row r="6" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="16" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="3">
         <v>0</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="9">
+      <c r="C6" s="8">
+        <v>5</v>
+      </c>
+      <c r="D6" s="8">
+        <v>5</v>
+      </c>
+      <c r="E6" s="8">
+        <v>5</v>
+      </c>
+      <c r="F6" s="8">
+        <v>5</v>
+      </c>
+      <c r="G6" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H6" s="9">
         <f>VLOOKUP(A6,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.15</v>
       </c>
-      <c r="E6" s="8">
+      <c r="I6" s="8">
         <v>3.15</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
+      <c r="J6" s="9">
+        <f t="shared" si="1"/>
+        <v>3.8899999999999997</v>
+      </c>
       <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
+      <c r="L6" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
@@ -22063,30 +22299,57 @@
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
       <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4"/>
+      <c r="AA6" s="4"/>
+      <c r="AB6" s="4"/>
+      <c r="AC6" s="4"/>
+      <c r="AD6" s="4"/>
+      <c r="AE6" s="4"/>
     </row>
-    <row r="7" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="3">
         <v>0</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="9">
+      <c r="C7" s="8">
+        <v>5</v>
+      </c>
+      <c r="D7" s="8">
+        <v>5</v>
+      </c>
+      <c r="E7" s="8">
+        <v>5</v>
+      </c>
+      <c r="F7" s="8">
+        <v>5</v>
+      </c>
+      <c r="G7" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H7" s="9">
         <f>VLOOKUP(A7,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.9499999999999997</v>
       </c>
-      <c r="E7" s="8">
+      <c r="I7" s="8">
         <v>3.9499999999999997</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
+      <c r="J7" s="9">
+        <f t="shared" si="1"/>
+        <v>4.3699999999999992</v>
+      </c>
       <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
+      <c r="L7" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M7" s="18">
+        <f>(6/7)*5</f>
+        <v>4.2857142857142856</v>
+      </c>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
@@ -22098,29 +22361,53 @@
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
       <c r="X7" s="4"/>
+      <c r="Y7" s="4"/>
+      <c r="Z7" s="4"/>
+      <c r="AA7" s="4"/>
+      <c r="AB7" s="4"/>
+      <c r="AC7" s="4"/>
+      <c r="AD7" s="4"/>
+      <c r="AE7" s="4"/>
     </row>
-    <row r="8" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="16" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="3">
         <v>0</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="9">
+      <c r="C8" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D8" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E8" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F8" s="8">
+        <v>3.8</v>
+      </c>
+      <c r="G8" s="9">
+        <f t="shared" si="0"/>
+        <v>4.1750000000000007</v>
+      </c>
+      <c r="H8" s="9">
         <f>VLOOKUP(A8,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>2.82</v>
       </c>
-      <c r="E8" s="9">
+      <c r="I8" s="9">
         <v>2.82</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
+      <c r="J8" s="9">
+        <f t="shared" si="1"/>
+        <v>3.3620000000000001</v>
+      </c>
       <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
+      <c r="L8" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
@@ -22133,32 +22420,58 @@
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
+      <c r="Y8" s="4"/>
+      <c r="Z8" s="4"/>
+      <c r="AA8" s="4"/>
+      <c r="AB8" s="4"/>
+      <c r="AC8" s="4"/>
+      <c r="AD8" s="4"/>
+      <c r="AE8" s="4"/>
     </row>
-    <row r="9" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="16" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="3">
         <v>0</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="9">
+      <c r="C9" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D9" s="8">
+        <v>5</v>
+      </c>
+      <c r="E9" s="8">
+        <v>5</v>
+      </c>
+      <c r="F9" s="8">
+        <v>5</v>
+      </c>
+      <c r="G9" s="9">
+        <f t="shared" si="0"/>
+        <v>4.8</v>
+      </c>
+      <c r="H9" s="9">
         <f>VLOOKUP(A9,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>2.82</v>
       </c>
-      <c r="E9" s="9">
+      <c r="I9" s="9">
         <v>2.82</v>
       </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
+      <c r="J9" s="9">
+        <f t="shared" si="1"/>
+        <v>3.6120000000000001</v>
+      </c>
       <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
+      <c r="L9" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
+      <c r="O9" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
@@ -22168,29 +22481,53 @@
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
+      <c r="Y9" s="4"/>
+      <c r="Z9" s="4"/>
+      <c r="AA9" s="4"/>
+      <c r="AB9" s="4"/>
+      <c r="AC9" s="4"/>
+      <c r="AD9" s="4"/>
+      <c r="AE9" s="4"/>
     </row>
-    <row r="10" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="16" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="3">
         <v>0</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="9">
+      <c r="C10" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D10" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E10" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F10" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="G10" s="9">
+        <f t="shared" si="0"/>
+        <v>4.3000000000000007</v>
+      </c>
+      <c r="H10" s="9">
         <f>VLOOKUP(A10,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>4.51</v>
       </c>
-      <c r="E10" s="8">
+      <c r="I10" s="8">
         <v>4.51</v>
       </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
+      <c r="J10" s="9">
+        <f t="shared" si="1"/>
+        <v>4.4260000000000002</v>
+      </c>
       <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
+      <c r="L10" s="8">
+        <f>IF(G10&lt;J10,1,0)</f>
+        <v>1</v>
+      </c>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
@@ -22203,29 +22540,53 @@
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
+      <c r="Y10" s="4"/>
+      <c r="Z10" s="4"/>
+      <c r="AA10" s="4"/>
+      <c r="AB10" s="4"/>
+      <c r="AC10" s="4"/>
+      <c r="AD10" s="4"/>
+      <c r="AE10" s="4"/>
     </row>
-    <row r="11" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="3">
         <v>6.25E-2</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="9">
+      <c r="C11" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D11" s="8">
+        <v>5</v>
+      </c>
+      <c r="E11" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F11" s="8">
+        <v>4</v>
+      </c>
+      <c r="G11" s="9">
+        <f t="shared" si="0"/>
+        <v>4.375</v>
+      </c>
+      <c r="H11" s="9">
         <f>VLOOKUP(A11,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.65</v>
       </c>
-      <c r="E11" s="8">
+      <c r="I11" s="8">
         <v>3.65</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
+      <c r="J11" s="9">
+        <f t="shared" si="1"/>
+        <v>3.94</v>
+      </c>
       <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
+      <c r="L11" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
@@ -22238,29 +22599,53 @@
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
       <c r="X11" s="4"/>
+      <c r="Y11" s="4"/>
+      <c r="Z11" s="4"/>
+      <c r="AA11" s="4"/>
+      <c r="AB11" s="4"/>
+      <c r="AC11" s="4"/>
+      <c r="AD11" s="4"/>
+      <c r="AE11" s="4"/>
     </row>
-    <row r="12" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="16" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="3">
         <v>0</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="9">
+      <c r="C12" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D12" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E12" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F12" s="8">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9">
+        <f t="shared" si="0"/>
+        <v>3.2250000000000005</v>
+      </c>
+      <c r="H12" s="9">
         <f>VLOOKUP(A12,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.64</v>
       </c>
-      <c r="E12" s="8">
+      <c r="I12" s="8">
         <v>3.64</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
+      <c r="J12" s="9">
+        <f t="shared" si="1"/>
+        <v>3.4740000000000002</v>
+      </c>
       <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
+      <c r="L12" s="8">
+        <f>IF(G12&lt;J12,1,0)</f>
+        <v>1</v>
+      </c>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
@@ -22273,29 +22658,53 @@
       <c r="V12" s="4"/>
       <c r="W12" s="4"/>
       <c r="X12" s="4"/>
+      <c r="Y12" s="4"/>
+      <c r="Z12" s="4"/>
+      <c r="AA12" s="4"/>
+      <c r="AB12" s="4"/>
+      <c r="AC12" s="4"/>
+      <c r="AD12" s="4"/>
+      <c r="AE12" s="4"/>
     </row>
-    <row r="13" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="16" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="3">
         <v>0</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="9">
+      <c r="C13" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D13" s="8">
+        <v>5</v>
+      </c>
+      <c r="E13" s="8">
+        <v>5</v>
+      </c>
+      <c r="F13" s="8">
+        <v>5</v>
+      </c>
+      <c r="G13" s="9">
+        <f t="shared" si="0"/>
+        <v>4.8</v>
+      </c>
+      <c r="H13" s="9">
         <f>VLOOKUP(A13,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.65</v>
       </c>
-      <c r="E13" s="8">
+      <c r="I13" s="8">
         <v>3.65</v>
       </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
+      <c r="J13" s="9">
+        <f t="shared" si="1"/>
+        <v>4.1099999999999994</v>
+      </c>
       <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
+      <c r="L13" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
@@ -22308,29 +22717,53 @@
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
       <c r="X13" s="4"/>
+      <c r="Y13" s="4"/>
+      <c r="Z13" s="4"/>
+      <c r="AA13" s="4"/>
+      <c r="AB13" s="4"/>
+      <c r="AC13" s="4"/>
+      <c r="AD13" s="4"/>
+      <c r="AE13" s="4"/>
     </row>
-    <row r="14" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B14" s="3">
         <v>0</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="9">
+      <c r="C14" s="8">
+        <v>5</v>
+      </c>
+      <c r="D14" s="8">
+        <v>5</v>
+      </c>
+      <c r="E14" s="8">
+        <v>5</v>
+      </c>
+      <c r="F14" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="G14" s="9">
+        <f t="shared" si="0"/>
+        <v>4.875</v>
+      </c>
+      <c r="H14" s="9">
         <f>VLOOKUP(A14,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>4.2799999999999994</v>
       </c>
-      <c r="E14" s="8">
+      <c r="I14" s="8">
         <v>4.2799999999999994</v>
       </c>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
+      <c r="J14" s="9">
+        <f t="shared" si="1"/>
+        <v>4.5179999999999998</v>
+      </c>
       <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
+      <c r="L14" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
@@ -22343,29 +22776,53 @@
       <c r="V14" s="4"/>
       <c r="W14" s="4"/>
       <c r="X14" s="4"/>
+      <c r="Y14" s="4"/>
+      <c r="Z14" s="4"/>
+      <c r="AA14" s="4"/>
+      <c r="AB14" s="4"/>
+      <c r="AC14" s="4"/>
+      <c r="AD14" s="4"/>
+      <c r="AE14" s="4"/>
     </row>
-    <row r="15" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B15" s="3">
         <v>0.125</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="9">
+      <c r="C15" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D15" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E15" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F15" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="G15" s="9">
+        <f t="shared" si="0"/>
+        <v>4.1000000000000005</v>
+      </c>
+      <c r="H15" s="9">
         <f>VLOOKUP(A15,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>1.26</v>
       </c>
-      <c r="E15" s="9">
+      <c r="I15" s="9">
         <v>1.26</v>
       </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
+      <c r="J15" s="9">
+        <f t="shared" si="1"/>
+        <v>2.3960000000000004</v>
+      </c>
       <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
+      <c r="L15" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
@@ -22378,29 +22835,53 @@
       <c r="V15" s="4"/>
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
+      <c r="Y15" s="4"/>
+      <c r="Z15" s="4"/>
+      <c r="AA15" s="4"/>
+      <c r="AB15" s="4"/>
+      <c r="AC15" s="4"/>
+      <c r="AD15" s="4"/>
+      <c r="AE15" s="4"/>
     </row>
-    <row r="16" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="16" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="3">
         <v>6.25E-2</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="9">
+      <c r="C16" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D16" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E16" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F16" s="8">
+        <v>3.8</v>
+      </c>
+      <c r="G16" s="9">
+        <f t="shared" si="0"/>
+        <v>4.1750000000000007</v>
+      </c>
+      <c r="H16" s="9">
         <f>VLOOKUP(A16,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>2.62</v>
       </c>
-      <c r="E16" s="9">
+      <c r="I16" s="9">
         <v>2.62</v>
       </c>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
+      <c r="J16" s="9">
+        <f t="shared" si="1"/>
+        <v>3.2420000000000004</v>
+      </c>
       <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
+      <c r="L16" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="4"/>
@@ -22413,29 +22894,53 @@
       <c r="V16" s="4"/>
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
+      <c r="Y16" s="4"/>
+      <c r="Z16" s="4"/>
+      <c r="AA16" s="4"/>
+      <c r="AB16" s="4"/>
+      <c r="AC16" s="4"/>
+      <c r="AD16" s="4"/>
+      <c r="AE16" s="4"/>
     </row>
-    <row r="17" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="16" t="s">
         <v>16</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="9">
+      <c r="C17" s="8">
+        <v>5</v>
+      </c>
+      <c r="D17" s="8">
+        <v>5</v>
+      </c>
+      <c r="E17" s="8">
+        <v>5</v>
+      </c>
+      <c r="F17" s="8">
+        <v>5</v>
+      </c>
+      <c r="G17" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H17" s="9">
         <f>VLOOKUP(A17,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>4.6099999999999994</v>
       </c>
-      <c r="E17" s="8">
+      <c r="I17" s="8">
         <v>4.6099999999999994</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
+      <c r="J17" s="9">
+        <f t="shared" si="1"/>
+        <v>4.766</v>
+      </c>
       <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
+      <c r="L17" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
@@ -22448,64 +22953,111 @@
       <c r="V17" s="4"/>
       <c r="W17" s="4"/>
       <c r="X17" s="4"/>
+      <c r="Y17" s="4"/>
+      <c r="Z17" s="4"/>
+      <c r="AA17" s="4"/>
+      <c r="AB17" s="4"/>
+      <c r="AC17" s="4"/>
+      <c r="AD17" s="4"/>
+      <c r="AE17" s="4"/>
     </row>
-    <row r="18" spans="1:24" s="15" customFormat="1" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="11" t="s">
+    <row r="18" spans="1:31" s="14" customFormat="1" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="11">
         <v>0.1875</v>
       </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14" t="e">
-        <f>VLOOKUP(A18,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E18" s="16" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="13"/>
-      <c r="S18" s="13"/>
-      <c r="T18" s="13"/>
-      <c r="U18" s="13"/>
-      <c r="V18" s="13"/>
-      <c r="W18" s="13"/>
-      <c r="X18" s="13"/>
+      <c r="C18" s="15">
+        <v>3</v>
+      </c>
+      <c r="D18" s="15">
+        <v>0</v>
+      </c>
+      <c r="E18" s="15">
+        <v>1</v>
+      </c>
+      <c r="F18" s="15">
+        <v>0</v>
+      </c>
+      <c r="G18" s="13">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H18" s="13">
+        <v>0</v>
+      </c>
+      <c r="I18" s="15">
+        <v>0</v>
+      </c>
+      <c r="J18" s="13">
+        <f t="shared" si="1"/>
+        <v>0.4</v>
+      </c>
+      <c r="K18" s="12"/>
+      <c r="L18" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="12"/>
+      <c r="U18" s="12"/>
+      <c r="V18" s="12"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="12"/>
+      <c r="Y18" s="12"/>
+      <c r="Z18" s="12"/>
+      <c r="AA18" s="12"/>
+      <c r="AB18" s="12"/>
+      <c r="AC18" s="12"/>
+      <c r="AD18" s="12"/>
+      <c r="AE18" s="12"/>
     </row>
-    <row r="19" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B19" s="3">
         <v>0</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="9">
+      <c r="C19" s="8">
+        <v>5</v>
+      </c>
+      <c r="D19" s="8">
+        <v>5</v>
+      </c>
+      <c r="E19" s="8">
+        <v>5</v>
+      </c>
+      <c r="F19" s="8">
+        <v>0</v>
+      </c>
+      <c r="G19" s="9">
+        <f t="shared" si="0"/>
+        <v>3.75</v>
+      </c>
+      <c r="H19" s="9">
         <f>VLOOKUP(A19,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>0.73</v>
       </c>
-      <c r="E19" s="9">
+      <c r="I19" s="9">
         <v>0.73</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
+      <c r="J19" s="9">
+        <f t="shared" si="1"/>
+        <v>1.9379999999999999</v>
+      </c>
       <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
+      <c r="L19" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M19" s="4"/>
       <c r="N19" s="4"/>
       <c r="O19" s="4"/>
@@ -22518,29 +23070,53 @@
       <c r="V19" s="4"/>
       <c r="W19" s="4"/>
       <c r="X19" s="4"/>
+      <c r="Y19" s="4"/>
+      <c r="Z19" s="4"/>
+      <c r="AA19" s="4"/>
+      <c r="AB19" s="4"/>
+      <c r="AC19" s="4"/>
+      <c r="AD19" s="4"/>
+      <c r="AE19" s="4"/>
     </row>
-    <row r="20" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="16" t="s">
         <v>19</v>
       </c>
       <c r="B20" s="3">
         <v>0</v>
       </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="9">
+      <c r="C20" s="8">
+        <v>5</v>
+      </c>
+      <c r="D20" s="8">
+        <v>5</v>
+      </c>
+      <c r="E20" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F20" s="8">
+        <v>5</v>
+      </c>
+      <c r="G20" s="9">
+        <f t="shared" si="0"/>
+        <v>4.8250000000000002</v>
+      </c>
+      <c r="H20" s="9">
         <f>VLOOKUP(A20,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.65</v>
       </c>
-      <c r="E20" s="8">
+      <c r="I20" s="8">
         <v>3.65</v>
       </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
+      <c r="J20" s="9">
+        <f t="shared" si="1"/>
+        <v>4.12</v>
+      </c>
       <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
+      <c r="L20" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
       <c r="O20" s="4"/>
@@ -22553,29 +23129,53 @@
       <c r="V20" s="4"/>
       <c r="W20" s="4"/>
       <c r="X20" s="4"/>
+      <c r="Y20" s="4"/>
+      <c r="Z20" s="4"/>
+      <c r="AA20" s="4"/>
+      <c r="AB20" s="4"/>
+      <c r="AC20" s="4"/>
+      <c r="AD20" s="4"/>
+      <c r="AE20" s="4"/>
     </row>
-    <row r="21" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="3">
         <v>0</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="9">
+      <c r="C21" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D21" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E21" s="8">
+        <v>5</v>
+      </c>
+      <c r="F21" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="G21" s="9">
+        <f t="shared" si="0"/>
+        <v>4.5250000000000004</v>
+      </c>
+      <c r="H21" s="9">
         <f>VLOOKUP(A21,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.25</v>
       </c>
-      <c r="E21" s="8">
+      <c r="I21" s="8">
         <v>3.25</v>
       </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
+      <c r="J21" s="9">
+        <f t="shared" si="1"/>
+        <v>3.7600000000000002</v>
+      </c>
       <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
+      <c r="L21" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
@@ -22588,33 +23188,58 @@
       <c r="V21" s="4"/>
       <c r="W21" s="4"/>
       <c r="X21" s="4"/>
+      <c r="Y21" s="4"/>
+      <c r="Z21" s="4"/>
+      <c r="AA21" s="4"/>
+      <c r="AB21" s="4"/>
+      <c r="AC21" s="4"/>
+      <c r="AD21" s="4"/>
+      <c r="AE21" s="4"/>
     </row>
-    <row r="22" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="16" t="s">
         <v>21</v>
       </c>
       <c r="B22" s="3">
         <v>0</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="9">
+      <c r="C22" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D22" s="8">
+        <v>5</v>
+      </c>
+      <c r="E22" s="8">
+        <v>5</v>
+      </c>
+      <c r="F22" s="8">
+        <v>5</v>
+      </c>
+      <c r="G22" s="9">
+        <f t="shared" si="0"/>
+        <v>4.8</v>
+      </c>
+      <c r="H22" s="9">
         <f>VLOOKUP(A22,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.6499999999999995</v>
       </c>
-      <c r="E22" s="8">
+      <c r="I22" s="8">
         <v>3.6499999999999995</v>
       </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
+      <c r="J22" s="9">
+        <f t="shared" si="1"/>
+        <v>4.1099999999999994</v>
+      </c>
       <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
+      <c r="L22" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
+      <c r="O22" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="Q22" s="4"/>
       <c r="R22" s="4"/>
       <c r="S22" s="4"/>
@@ -22623,29 +23248,53 @@
       <c r="V22" s="4"/>
       <c r="W22" s="4"/>
       <c r="X22" s="4"/>
+      <c r="Y22" s="4"/>
+      <c r="Z22" s="4"/>
+      <c r="AA22" s="4"/>
+      <c r="AB22" s="4"/>
+      <c r="AC22" s="4"/>
+      <c r="AD22" s="4"/>
+      <c r="AE22" s="4"/>
     </row>
-    <row r="23" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="16" t="s">
         <v>22</v>
       </c>
       <c r="B23" s="3">
         <v>0</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="9">
+      <c r="C23" s="8">
+        <v>5</v>
+      </c>
+      <c r="D23" s="8">
+        <v>5</v>
+      </c>
+      <c r="E23" s="8">
+        <v>5</v>
+      </c>
+      <c r="F23" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="G23" s="9">
+        <f t="shared" si="0"/>
+        <v>4.875</v>
+      </c>
+      <c r="H23" s="9">
         <f>VLOOKUP(A23,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.3499999999999996</v>
       </c>
-      <c r="E23" s="8">
+      <c r="I23" s="8">
         <v>3.3499999999999996</v>
       </c>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
+      <c r="J23" s="9">
+        <f t="shared" si="1"/>
+        <v>3.96</v>
+      </c>
       <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
+      <c r="L23" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M23" s="4"/>
       <c r="N23" s="4"/>
       <c r="O23" s="4"/>
@@ -22658,30 +23307,57 @@
       <c r="V23" s="4"/>
       <c r="W23" s="4"/>
       <c r="X23" s="4"/>
+      <c r="Y23" s="4"/>
+      <c r="Z23" s="4"/>
+      <c r="AA23" s="4"/>
+      <c r="AB23" s="4"/>
+      <c r="AC23" s="4"/>
+      <c r="AD23" s="4"/>
+      <c r="AE23" s="4"/>
     </row>
-    <row r="24" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="16" t="s">
         <v>23</v>
       </c>
       <c r="B24" s="3">
         <v>0</v>
       </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="9">
+      <c r="C24" s="8">
+        <v>5</v>
+      </c>
+      <c r="D24" s="8">
+        <v>5</v>
+      </c>
+      <c r="E24" s="8">
+        <v>5</v>
+      </c>
+      <c r="F24" s="8">
+        <v>5</v>
+      </c>
+      <c r="G24" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H24" s="9">
         <f>VLOOKUP(A24,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.02</v>
       </c>
-      <c r="E24" s="8">
+      <c r="I24" s="8">
         <v>3.02</v>
       </c>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
+      <c r="J24" s="9">
+        <f t="shared" si="1"/>
+        <v>3.8119999999999998</v>
+      </c>
       <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
-      <c r="M24" s="4"/>
+      <c r="L24" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="8">
+        <f>(5/8)*7</f>
+        <v>4.375</v>
+      </c>
       <c r="N24" s="4"/>
       <c r="O24" s="4"/>
       <c r="P24" s="4"/>
@@ -22693,29 +23369,53 @@
       <c r="V24" s="4"/>
       <c r="W24" s="4"/>
       <c r="X24" s="4"/>
+      <c r="Y24" s="4"/>
+      <c r="Z24" s="4"/>
+      <c r="AA24" s="4"/>
+      <c r="AB24" s="4"/>
+      <c r="AC24" s="4"/>
+      <c r="AD24" s="4"/>
+      <c r="AE24" s="4"/>
     </row>
-    <row r="25" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="16" t="s">
         <v>24</v>
       </c>
       <c r="B25" s="3">
         <v>0</v>
       </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="9">
+      <c r="C25" s="8">
+        <v>5</v>
+      </c>
+      <c r="D25" s="8">
+        <v>5</v>
+      </c>
+      <c r="E25" s="8">
+        <v>5</v>
+      </c>
+      <c r="F25" s="8">
+        <v>5</v>
+      </c>
+      <c r="G25" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H25" s="9">
         <f>VLOOKUP(A25,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.4499999999999997</v>
       </c>
-      <c r="E25" s="8">
+      <c r="I25" s="8">
         <v>3.4499999999999997</v>
       </c>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
+      <c r="J25" s="9">
+        <f t="shared" si="1"/>
+        <v>4.07</v>
+      </c>
       <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
+      <c r="L25" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M25" s="4"/>
       <c r="N25" s="4"/>
       <c r="O25" s="4"/>
@@ -22728,29 +23428,53 @@
       <c r="V25" s="4"/>
       <c r="W25" s="4"/>
       <c r="X25" s="4"/>
+      <c r="Y25" s="4"/>
+      <c r="Z25" s="4"/>
+      <c r="AA25" s="4"/>
+      <c r="AB25" s="4"/>
+      <c r="AC25" s="4"/>
+      <c r="AD25" s="4"/>
+      <c r="AE25" s="4"/>
     </row>
-    <row r="26" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="16" t="s">
         <v>25</v>
       </c>
       <c r="B26" s="3">
         <v>6.25E-2</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="9">
+      <c r="C26" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D26" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E26" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="F26" s="8">
+        <v>0</v>
+      </c>
+      <c r="G26" s="9">
+        <f t="shared" si="0"/>
+        <v>3.2250000000000005</v>
+      </c>
+      <c r="H26" s="9">
         <f>VLOOKUP(A26,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E26" s="9">
+      <c r="I26" s="9">
         <v>0</v>
       </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
+      <c r="J26" s="9">
+        <f t="shared" si="1"/>
+        <v>1.2900000000000003</v>
+      </c>
       <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
+      <c r="L26" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M26" s="4"/>
       <c r="N26" s="4"/>
       <c r="O26" s="4"/>
@@ -22763,29 +23487,53 @@
       <c r="V26" s="4"/>
       <c r="W26" s="4"/>
       <c r="X26" s="4"/>
+      <c r="Y26" s="4"/>
+      <c r="Z26" s="4"/>
+      <c r="AA26" s="4"/>
+      <c r="AB26" s="4"/>
+      <c r="AC26" s="4"/>
+      <c r="AD26" s="4"/>
+      <c r="AE26" s="4"/>
     </row>
-    <row r="27" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="16" t="s">
         <v>26</v>
       </c>
       <c r="B27" s="3">
         <v>0</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="9">
+      <c r="C27" s="8">
+        <v>5</v>
+      </c>
+      <c r="D27" s="8">
+        <v>5</v>
+      </c>
+      <c r="E27" s="8">
+        <v>5</v>
+      </c>
+      <c r="F27" s="8">
+        <v>5</v>
+      </c>
+      <c r="G27" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H27" s="9">
         <f>VLOOKUP(A27,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>2.48</v>
       </c>
-      <c r="E27" s="9">
+      <c r="I27" s="9">
         <v>2.48</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
+      <c r="J27" s="9">
+        <f t="shared" si="1"/>
+        <v>3.488</v>
+      </c>
       <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
+      <c r="L27" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
       <c r="O27" s="4"/>
@@ -22798,29 +23546,53 @@
       <c r="V27" s="4"/>
       <c r="W27" s="4"/>
       <c r="X27" s="4"/>
+      <c r="Y27" s="4"/>
+      <c r="Z27" s="4"/>
+      <c r="AA27" s="4"/>
+      <c r="AB27" s="4"/>
+      <c r="AC27" s="4"/>
+      <c r="AD27" s="4"/>
+      <c r="AE27" s="4"/>
     </row>
-    <row r="28" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="16" t="s">
         <v>27</v>
       </c>
       <c r="B28" s="3">
         <v>0</v>
       </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="9">
+      <c r="C28" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D28" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="E28" s="8">
+        <v>5</v>
+      </c>
+      <c r="F28" s="8">
+        <v>4</v>
+      </c>
+      <c r="G28" s="9">
+        <f t="shared" si="0"/>
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="H28" s="9">
         <f>VLOOKUP(A28,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>4.41</v>
       </c>
-      <c r="E28" s="8">
+      <c r="I28" s="8">
         <v>4.41</v>
       </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
+      <c r="J28" s="9">
+        <f t="shared" si="1"/>
+        <v>4.4060000000000006</v>
+      </c>
       <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
+      <c r="L28" s="8">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
@@ -22833,29 +23605,53 @@
       <c r="V28" s="4"/>
       <c r="W28" s="4"/>
       <c r="X28" s="4"/>
+      <c r="Y28" s="4"/>
+      <c r="Z28" s="4"/>
+      <c r="AA28" s="4"/>
+      <c r="AB28" s="4"/>
+      <c r="AC28" s="4"/>
+      <c r="AD28" s="4"/>
+      <c r="AE28" s="4"/>
     </row>
-    <row r="29" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
+    <row r="29" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="16" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="3">
         <v>0</v>
       </c>
-      <c r="C29" s="4"/>
-      <c r="D29" s="9">
+      <c r="C29" s="8">
+        <v>5</v>
+      </c>
+      <c r="D29" s="8">
+        <v>5</v>
+      </c>
+      <c r="E29" s="8">
+        <v>5</v>
+      </c>
+      <c r="F29" s="8">
+        <v>5</v>
+      </c>
+      <c r="G29" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H29" s="9">
         <f>VLOOKUP(A29,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>2.72</v>
       </c>
-      <c r="E29" s="9">
+      <c r="I29" s="9">
         <v>2.72</v>
       </c>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
+      <c r="J29" s="9">
+        <f t="shared" si="1"/>
+        <v>3.6320000000000001</v>
+      </c>
       <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
+      <c r="L29" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M29" s="4"/>
       <c r="N29" s="4"/>
       <c r="O29" s="4"/>
@@ -22868,29 +23664,53 @@
       <c r="V29" s="4"/>
       <c r="W29" s="4"/>
       <c r="X29" s="4"/>
+      <c r="Y29" s="4"/>
+      <c r="Z29" s="4"/>
+      <c r="AA29" s="4"/>
+      <c r="AB29" s="4"/>
+      <c r="AC29" s="4"/>
+      <c r="AD29" s="4"/>
+      <c r="AE29" s="4"/>
     </row>
-    <row r="30" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+    <row r="30" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="16" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="3">
         <v>0</v>
       </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="9">
+      <c r="C30" s="8">
+        <v>5</v>
+      </c>
+      <c r="D30" s="8">
+        <v>5</v>
+      </c>
+      <c r="E30" s="8">
+        <v>5</v>
+      </c>
+      <c r="F30" s="8">
+        <v>5</v>
+      </c>
+      <c r="G30" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H30" s="9">
         <f>VLOOKUP(A30,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>2.09</v>
       </c>
-      <c r="E30" s="9">
+      <c r="I30" s="9">
         <v>2.09</v>
       </c>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
+      <c r="J30" s="9">
+        <f t="shared" si="1"/>
+        <v>3.2539999999999996</v>
+      </c>
       <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
+      <c r="L30" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M30" s="4"/>
       <c r="N30" s="4"/>
       <c r="O30" s="4"/>
@@ -22903,29 +23723,53 @@
       <c r="V30" s="4"/>
       <c r="W30" s="4"/>
       <c r="X30" s="4"/>
+      <c r="Y30" s="4"/>
+      <c r="Z30" s="4"/>
+      <c r="AA30" s="4"/>
+      <c r="AB30" s="4"/>
+      <c r="AC30" s="4"/>
+      <c r="AD30" s="4"/>
+      <c r="AE30" s="4"/>
     </row>
-    <row r="31" spans="1:24" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+    <row r="31" spans="1:31" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="16" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="3">
         <v>0</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="9">
+      <c r="C31" s="8">
+        <v>5</v>
+      </c>
+      <c r="D31" s="8">
+        <v>5</v>
+      </c>
+      <c r="E31" s="8">
+        <v>5</v>
+      </c>
+      <c r="F31" s="8">
+        <v>5</v>
+      </c>
+      <c r="G31" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H31" s="9">
         <f>VLOOKUP(A31,'Quiz 1_Consolidado'!$A$2:$B$30,2,FALSE)</f>
         <v>3.6499999999999995</v>
       </c>
-      <c r="E31" s="8">
+      <c r="I31" s="8">
         <v>3.6499999999999995</v>
       </c>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
+      <c r="J31" s="9">
+        <f t="shared" si="1"/>
+        <v>4.1899999999999995</v>
+      </c>
       <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
+      <c r="L31" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
       <c r="M31" s="4"/>
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
@@ -22938,12 +23782,19 @@
       <c r="V31" s="4"/>
       <c r="W31" s="4"/>
       <c r="X31" s="4"/>
+      <c r="Y31" s="4"/>
+      <c r="Z31" s="4"/>
+      <c r="AA31" s="4"/>
+      <c r="AB31" s="4"/>
+      <c r="AC31" s="4"/>
+      <c r="AD31" s="4"/>
+      <c r="AE31" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="D1:E31" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>